<commit_message>
#26 Deliverables Done. Client BOM Remaining.
</commit_message>
<xml_diff>
--- a/Design Files/Solenoid-Switching-Board-v1.0/BOM/Client BOM.xlsx
+++ b/Design Files/Solenoid-Switching-Board-v1.0/BOM/Client BOM.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LiberDB\Documents\GitHub\muhunthancanagey-servocontrol\Design Files\Solenoid-Switching-Board-v1.0\Project Outputs for Solenoid-Switching-Board-v1.0\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LiberDB\Documents\GitHub\muhunthancanagey-servocontrol\Design Files\Solenoid-Switching-Board-v1.0\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -1354,14 +1354,14 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1674,9 +1674,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2787,7 +2787,7 @@
       <c r="H36" s="9" t="s">
         <v>308</v>
       </c>
-      <c r="I36" s="15" t="s">
+      <c r="I36" s="14" t="s">
         <v>372</v>
       </c>
       <c r="J36" s="9">
@@ -3369,7 +3369,7 @@
       <c r="J54" s="9">
         <v>2</v>
       </c>
-      <c r="K54" s="16" t="s">
+      <c r="K54" s="15" t="s">
         <v>333</v>
       </c>
     </row>
@@ -3785,7 +3785,7 @@
       <c r="J67" s="7">
         <v>1</v>
       </c>
-      <c r="K67" s="16" t="s">
+      <c r="K67" s="15" t="s">
         <v>333</v>
       </c>
     </row>
@@ -4203,7 +4203,7 @@
       <c r="J80" s="9">
         <v>1</v>
       </c>
-      <c r="K80" s="16" t="s">
+      <c r="K80" s="15" t="s">
         <v>333</v>
       </c>
     </row>

</xml_diff>

<commit_message>
#26 Client BOM added
</commit_message>
<xml_diff>
--- a/Design Files/Solenoid-Switching-Board-v1.0/BOM/Client BOM.xlsx
+++ b/Design Files/Solenoid-Switching-Board-v1.0/BOM/Client BOM.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LiberDB\Documents\GitHub\muhunthancanagey-servocontrol\Design Files\Solenoid-Switching-Board-v1.0\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iftikhar Ahmed\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="372">
   <si>
     <t>#</t>
   </si>
@@ -603,9 +603,6 @@
     <t>IND-0402</t>
   </si>
   <si>
-    <t>TYPE-C-31-M-12_</t>
-  </si>
-  <si>
     <t>HDR 1x8 TH male</t>
   </si>
   <si>
@@ -678,9 +675,6 @@
     <t>MC-306</t>
   </si>
   <si>
-    <t>5TJ480000XYLBC_</t>
-  </si>
-  <si>
     <t>SMD3225-4P</t>
   </si>
   <si>
@@ -1128,29 +1122,26 @@
     <t>Quantity</t>
   </si>
   <si>
-    <t>Terminal</t>
+    <t>-------</t>
   </si>
   <si>
     <t>Value</t>
   </si>
   <si>
-    <t>Remarks</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>10 Ohm</t>
-  </si>
-  <si>
-    <t>600  Ohm</t>
+    <t xml:space="preserve"> Remarks</t>
+  </si>
+  <si>
+    <t>Custom</t>
+  </si>
+  <si>
+    <t>DO NOT PLACE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1194,8 +1185,17 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <strike/>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
-      <sz val="9"/>
+      <strike/>
+      <sz val="10"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1317,7 +1317,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1354,14 +1354,20 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1650,7 +1656,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K83"/>
+  <dimension ref="A1:K82"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
@@ -1660,9 +1666,9 @@
     <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1674,9 +1680,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1696,19 +1702,19 @@
         <v>179</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1730,13 +1736,13 @@
         <v>180</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J3" s="7">
         <v>11</v>
@@ -1759,16 +1765,16 @@
         <v>103</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>181</v>
+        <v>370</v>
       </c>
       <c r="G4" s="10" t="s">
         <v>181</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="J4" s="9">
         <v>2</v>
@@ -1794,13 +1800,13 @@
         <v>182</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="J5" s="7">
         <v>2</v>
@@ -1826,13 +1832,13 @@
         <v>183</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="J6" s="9">
         <v>1</v>
@@ -1858,13 +1864,13 @@
         <v>183</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="J7" s="7">
         <v>2</v>
@@ -1880,28 +1886,30 @@
       <c r="C8" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="17" t="s">
         <v>105</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="G8" s="10" t="s">
-        <v>224</v>
-      </c>
-      <c r="H8" s="9" t="s">
-        <v>292</v>
-      </c>
-      <c r="I8" s="10" t="s">
-        <v>333</v>
-      </c>
-      <c r="J8" s="9">
+      <c r="G8" s="17" t="s">
+        <v>222</v>
+      </c>
+      <c r="H8" s="16" t="s">
+        <v>290</v>
+      </c>
+      <c r="I8" s="17" t="s">
+        <v>331</v>
+      </c>
+      <c r="J8" s="16">
         <v>2</v>
       </c>
-      <c r="K8" s="9"/>
+      <c r="K8" s="18" t="s">
+        <v>371</v>
+      </c>
     </row>
     <row r="9" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1922,13 +1930,13 @@
         <v>182</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -1954,13 +1962,13 @@
         <v>183</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="J10" s="9">
         <v>5</v>
@@ -1986,13 +1994,13 @@
         <v>183</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="J11" s="7">
         <v>2</v>
@@ -2018,13 +2026,13 @@
         <v>183</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="J12" s="9">
         <v>2</v>
@@ -2050,13 +2058,13 @@
         <v>183</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="J13" s="7">
         <v>7</v>
@@ -2082,13 +2090,13 @@
         <v>183</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="J14" s="9">
         <v>4</v>
@@ -2114,13 +2122,13 @@
         <v>182</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
@@ -2146,13 +2154,13 @@
         <v>183</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="J16" s="9">
         <v>2</v>
@@ -2168,28 +2176,28 @@
       <c r="C17" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="F17" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="G17" s="8" t="s">
-        <v>234</v>
-      </c>
-      <c r="H17" s="7" t="s">
-        <v>293</v>
-      </c>
-      <c r="I17" s="8" t="s">
-        <v>333</v>
-      </c>
-      <c r="J17" s="7">
+      <c r="G17" s="17" t="s">
+        <v>232</v>
+      </c>
+      <c r="H17" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="I17" s="17" t="s">
+        <v>331</v>
+      </c>
+      <c r="J17" s="16">
         <v>8</v>
       </c>
-      <c r="K17" s="7"/>
+      <c r="K17" s="18"/>
     </row>
     <row r="18" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
@@ -2210,13 +2218,13 @@
         <v>183</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="J18" s="9">
         <v>2</v>
@@ -2242,13 +2250,13 @@
         <v>184</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="J19" s="7">
         <v>3</v>
@@ -2274,13 +2282,13 @@
         <v>185</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>296</v>
-      </c>
-      <c r="I20" s="10" t="s">
-        <v>372</v>
+        <v>294</v>
+      </c>
+      <c r="I20" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
@@ -2306,13 +2314,13 @@
         <v>186</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>297</v>
-      </c>
-      <c r="I21" s="8" t="s">
-        <v>372</v>
+        <v>295</v>
+      </c>
+      <c r="I21" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J21" s="7">
         <v>2</v>
@@ -2338,13 +2346,13 @@
         <v>187</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>298</v>
-      </c>
-      <c r="I22" s="10" t="s">
-        <v>372</v>
+        <v>296</v>
+      </c>
+      <c r="I22" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J22" s="9">
         <v>2</v>
@@ -2370,13 +2378,13 @@
         <v>188</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>299</v>
-      </c>
-      <c r="I23" s="8" t="s">
-        <v>372</v>
+        <v>297</v>
+      </c>
+      <c r="I23" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J23" s="7">
         <v>2</v>
@@ -2402,13 +2410,13 @@
         <v>189</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>300</v>
-      </c>
-      <c r="I24" s="10" t="s">
-        <v>372</v>
+        <v>298</v>
+      </c>
+      <c r="I24" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J24" s="9">
         <v>1</v>
@@ -2434,13 +2442,13 @@
         <v>190</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>301</v>
-      </c>
-      <c r="I25" s="8" t="s">
-        <v>372</v>
+        <v>299</v>
+      </c>
+      <c r="I25" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J25" s="7">
         <v>2</v>
@@ -2466,13 +2474,13 @@
         <v>191</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>302</v>
-      </c>
-      <c r="I26" s="10" t="s">
-        <v>372</v>
+        <v>300</v>
+      </c>
+      <c r="I26" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J26" s="9">
         <v>2</v>
@@ -2498,13 +2506,13 @@
         <v>185</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>303</v>
-      </c>
-      <c r="I27" s="8" t="s">
-        <v>372</v>
+        <v>301</v>
+      </c>
+      <c r="I27" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J27" s="7">
         <v>16</v>
@@ -2530,13 +2538,13 @@
         <v>192</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>304</v>
-      </c>
-      <c r="I28" s="10" t="s">
-        <v>372</v>
+        <v>302</v>
+      </c>
+      <c r="I28" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J28" s="9">
         <v>6</v>
@@ -2562,13 +2570,13 @@
         <v>193</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>293</v>
-      </c>
-      <c r="I29" s="8" t="s">
-        <v>373</v>
+        <v>291</v>
+      </c>
+      <c r="I29" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J29" s="7">
         <v>2</v>
@@ -2597,10 +2605,10 @@
         <v>1715721</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>305</v>
-      </c>
-      <c r="I30" s="10" t="s">
-        <v>372</v>
+        <v>303</v>
+      </c>
+      <c r="I30" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J30" s="9">
         <v>4</v>
@@ -2622,17 +2630,17 @@
       <c r="E31" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="F31" s="7" t="s">
-        <v>194</v>
+      <c r="F31" s="9" t="s">
+        <v>370</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>306</v>
-      </c>
-      <c r="I31" s="8" t="s">
-        <v>372</v>
+        <v>304</v>
+      </c>
+      <c r="I31" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J31" s="7">
         <v>1</v>
@@ -2655,23 +2663,23 @@
         <v>130</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>307</v>
-      </c>
-      <c r="I32" s="10" t="s">
-        <v>372</v>
+        <v>305</v>
+      </c>
+      <c r="I32" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>
       </c>
       <c r="K32" s="9"/>
     </row>
-    <row r="33" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="11">
         <f>ROW(B33) - ROW($B$2)</f>
@@ -2687,16 +2695,16 @@
         <v>131</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>307</v>
-      </c>
-      <c r="I33" s="8" t="s">
-        <v>372</v>
+        <v>305</v>
+      </c>
+      <c r="I33" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
@@ -2719,19 +2727,19 @@
         <v>132</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G34" s="10"/>
       <c r="H34" s="9"/>
-      <c r="I34" s="10" t="s">
-        <v>372</v>
+      <c r="I34" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
       </c>
       <c r="K34" s="9"/>
     </row>
-    <row r="35" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="11">
         <f>ROW(B35) - ROW($B$2)</f>
@@ -2747,16 +2755,16 @@
         <v>133</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>307</v>
-      </c>
-      <c r="I35" s="8" t="s">
-        <v>372</v>
+        <v>305</v>
+      </c>
+      <c r="I35" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J35" s="7">
         <v>1</v>
@@ -2779,16 +2787,16 @@
         <v>134</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>199</v>
+        <v>370</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>308</v>
-      </c>
-      <c r="I36" s="14" t="s">
-        <v>372</v>
+        <v>306</v>
+      </c>
+      <c r="I36" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J36" s="9">
         <v>4</v>
@@ -2810,17 +2818,17 @@
       <c r="E37" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="F37" s="7" t="s">
-        <v>200</v>
+      <c r="F37" s="9" t="s">
+        <v>370</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="H37" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="I37" s="8" t="s">
-        <v>372</v>
+        <v>307</v>
+      </c>
+      <c r="I37" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J37" s="7">
         <v>2</v>
@@ -2843,16 +2851,16 @@
         <v>136</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>201</v>
+        <v>370</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>310</v>
-      </c>
-      <c r="I38" s="10" t="s">
-        <v>372</v>
+        <v>308</v>
+      </c>
+      <c r="I38" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J38" s="9">
         <v>1</v>
@@ -2874,17 +2882,17 @@
       <c r="E39" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="F39" s="7" t="s">
-        <v>202</v>
+      <c r="F39" s="9" t="s">
+        <v>370</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="H39" s="7" t="s">
-        <v>311</v>
-      </c>
-      <c r="I39" s="8" t="s">
-        <v>372</v>
+        <v>309</v>
+      </c>
+      <c r="I39" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J39" s="7">
         <v>1</v>
@@ -2897,8 +2905,8 @@
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="C40" s="13" t="s">
-        <v>369</v>
+      <c r="C40" s="12" t="s">
+        <v>9</v>
       </c>
       <c r="D40" s="9" t="s">
         <v>58</v>
@@ -2907,16 +2915,16 @@
         <v>138</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>203</v>
+        <v>370</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>312</v>
-      </c>
-      <c r="I40" s="10" t="s">
-        <v>372</v>
+        <v>310</v>
+      </c>
+      <c r="I40" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J40" s="9">
         <v>1</v>
@@ -2938,17 +2946,17 @@
       <c r="E41" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="F41" s="7" t="s">
-        <v>204</v>
+      <c r="F41" s="9" t="s">
+        <v>370</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H41" s="7" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="I41" s="8" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="J41" s="7">
         <v>1</v>
@@ -2974,13 +2982,13 @@
         <v>193</v>
       </c>
       <c r="G42" s="10" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="I42" s="10" t="s">
-        <v>374</v>
+        <v>291</v>
+      </c>
+      <c r="I42" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J42" s="9">
         <v>1</v>
@@ -3003,16 +3011,16 @@
         <v>141</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="H43" s="7" t="s">
-        <v>314</v>
-      </c>
-      <c r="I43" s="8" t="s">
-        <v>372</v>
+        <v>312</v>
+      </c>
+      <c r="I43" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J43" s="7">
         <v>4</v>
@@ -3035,16 +3043,16 @@
         <v>142</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="G44" s="10" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>314</v>
-      </c>
-      <c r="I44" s="10" t="s">
-        <v>372</v>
+        <v>312</v>
+      </c>
+      <c r="I44" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J44" s="9">
         <v>1</v>
@@ -3067,16 +3075,16 @@
         <v>143</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>314</v>
-      </c>
-      <c r="I45" s="8" t="s">
-        <v>372</v>
+        <v>312</v>
+      </c>
+      <c r="I45" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J45" s="7">
         <v>16</v>
@@ -3099,16 +3107,16 @@
         <v>144</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="G46" s="10" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="H46" s="9" t="s">
-        <v>300</v>
-      </c>
-      <c r="I46" s="10" t="s">
-        <v>372</v>
+        <v>298</v>
+      </c>
+      <c r="I46" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J46" s="9">
         <v>16</v>
@@ -3131,16 +3139,16 @@
         <v>145</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="I47" s="8" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="J47" s="7">
         <v>1</v>
@@ -3163,16 +3171,16 @@
         <v>146</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G48" s="10" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="H48" s="9" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="I48" s="10" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="J48" s="9">
         <v>1</v>
@@ -3195,16 +3203,16 @@
         <v>147</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="H49" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I49" s="8" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="J49" s="7">
         <v>1</v>
@@ -3227,16 +3235,16 @@
         <v>148</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G50" s="10" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="H50" s="9" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="I50" s="10" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="J50" s="9">
         <v>1</v>
@@ -3259,16 +3267,16 @@
         <v>149</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="H51" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I51" s="8" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="J51" s="7">
         <v>1</v>
@@ -3291,16 +3299,16 @@
         <v>150</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G52" s="10" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="H52" s="9" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I52" s="10" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="J52" s="9">
         <v>1</v>
@@ -3323,16 +3331,16 @@
         <v>151</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="H53" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I53" s="8" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="J53" s="7">
         <v>17</v>
@@ -3348,30 +3356,28 @@
       <c r="C54" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D54" s="9" t="s">
+      <c r="D54" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="E54" s="10" t="s">
+      <c r="E54" s="17" t="s">
         <v>152</v>
       </c>
-      <c r="F54" s="9" t="s">
-        <v>208</v>
-      </c>
-      <c r="G54" s="10" t="s">
-        <v>263</v>
-      </c>
-      <c r="H54" s="9" t="s">
-        <v>292</v>
-      </c>
-      <c r="I54" s="10" t="s">
-        <v>333</v>
-      </c>
-      <c r="J54" s="9">
+      <c r="F54" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="G54" s="17" t="s">
+        <v>261</v>
+      </c>
+      <c r="H54" s="16" t="s">
+        <v>290</v>
+      </c>
+      <c r="I54" s="17" t="s">
+        <v>331</v>
+      </c>
+      <c r="J54" s="16">
         <v>2</v>
       </c>
-      <c r="K54" s="15" t="s">
-        <v>333</v>
-      </c>
+      <c r="K54" s="18"/>
     </row>
     <row r="55" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
@@ -3379,7 +3385,7 @@
         <f>ROW(B55) - ROW($B$2)</f>
         <v>53</v>
       </c>
-      <c r="C55" s="12" t="s">
+      <c r="C55" s="13" t="s">
         <v>14</v>
       </c>
       <c r="D55" s="7" t="s">
@@ -3389,16 +3395,16 @@
         <v>153</v>
       </c>
       <c r="F55" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G55" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="H55" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I55" s="8" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="J55" s="7">
         <v>2</v>
@@ -3421,16 +3427,16 @@
         <v>154</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G56" s="10" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="H56" s="9" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I56" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J56" s="9">
         <v>1</v>
@@ -3443,7 +3449,7 @@
         <f>ROW(B57) - ROW($B$2)</f>
         <v>55</v>
       </c>
-      <c r="C57" s="12" t="s">
+      <c r="C57" s="13" t="s">
         <v>14</v>
       </c>
       <c r="D57" s="7" t="s">
@@ -3453,16 +3459,16 @@
         <v>152</v>
       </c>
       <c r="F57" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G57" s="8" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="H57" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I57" s="8" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="J57" s="7">
         <v>2</v>
@@ -3485,16 +3491,16 @@
         <v>155</v>
       </c>
       <c r="F58" s="9" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G58" s="10" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="H58" s="9" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I58" s="10" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="J58" s="9">
         <v>24</v>
@@ -3507,7 +3513,7 @@
         <f>ROW(B59) - ROW($B$2)</f>
         <v>57</v>
       </c>
-      <c r="C59" s="12" t="s">
+      <c r="C59" s="13" t="s">
         <v>14</v>
       </c>
       <c r="D59" s="7" t="s">
@@ -3517,16 +3523,16 @@
         <v>156</v>
       </c>
       <c r="F59" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G59" s="8" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="H59" s="7" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="I59" s="8" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="J59" s="7">
         <v>1</v>
@@ -3539,7 +3545,7 @@
         <f t="shared" si="0"/>
         <v>58</v>
       </c>
-      <c r="C60" s="12" t="s">
+      <c r="C60" s="13" t="s">
         <v>14</v>
       </c>
       <c r="D60" s="9" t="s">
@@ -3549,14 +3555,14 @@
         <v>157</v>
       </c>
       <c r="F60" s="9" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G60" s="10" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="H60" s="9"/>
       <c r="I60" s="10" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="J60" s="9">
         <v>2</v>
@@ -3579,16 +3585,16 @@
         <v>158</v>
       </c>
       <c r="F61" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G61" s="8" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="H61" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I61" s="8" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="J61" s="7">
         <v>1</v>
@@ -3611,16 +3617,16 @@
         <v>159</v>
       </c>
       <c r="F62" s="9" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G62" s="10" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="H62" s="9" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I62" s="10" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="J62" s="9">
         <v>13</v>
@@ -3643,16 +3649,16 @@
         <v>160</v>
       </c>
       <c r="F63" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="G63" s="8" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="H63" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I63" s="8" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="J63" s="7">
         <v>6</v>
@@ -3675,16 +3681,16 @@
         <v>161</v>
       </c>
       <c r="F64" s="9" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G64" s="10" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="H64" s="9" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I64" s="10" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="J64" s="9">
         <v>2</v>
@@ -3707,16 +3713,16 @@
         <v>162</v>
       </c>
       <c r="F65" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G65" s="8" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="H65" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I65" s="8" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="J65" s="7">
         <v>2</v>
@@ -3739,16 +3745,16 @@
         <v>163</v>
       </c>
       <c r="F66" s="9" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G66" s="10" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="H66" s="9" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I66" s="10" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="J66" s="9">
         <v>1</v>
@@ -3764,30 +3770,28 @@
       <c r="C67" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D67" s="7" t="s">
+      <c r="D67" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="E67" s="8" t="s">
+      <c r="E67" s="17" t="s">
         <v>159</v>
       </c>
-      <c r="F67" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="G67" s="8" t="s">
-        <v>270</v>
-      </c>
-      <c r="H67" s="7" t="s">
-        <v>292</v>
-      </c>
-      <c r="I67" s="8" t="s">
-        <v>333</v>
-      </c>
-      <c r="J67" s="7">
+      <c r="F67" s="16" t="s">
+        <v>206</v>
+      </c>
+      <c r="G67" s="17" t="s">
+        <v>268</v>
+      </c>
+      <c r="H67" s="16" t="s">
+        <v>290</v>
+      </c>
+      <c r="I67" s="17" t="s">
+        <v>331</v>
+      </c>
+      <c r="J67" s="16">
         <v>1</v>
       </c>
-      <c r="K67" s="15" t="s">
-        <v>333</v>
-      </c>
+      <c r="K67" s="18"/>
     </row>
     <row r="68" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1"/>
@@ -3805,16 +3809,16 @@
         <v>164</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G68" s="10" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="H68" s="9" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I68" s="10" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="J68" s="9">
         <v>8</v>
@@ -3837,16 +3841,16 @@
         <v>165</v>
       </c>
       <c r="F69" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G69" s="8" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="H69" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I69" s="8" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="J69" s="7">
         <v>2</v>
@@ -3869,16 +3873,16 @@
         <v>166</v>
       </c>
       <c r="F70" s="9" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G70" s="10" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="H70" s="9" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I70" s="10" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="J70" s="9">
         <v>2</v>
@@ -3901,16 +3905,16 @@
         <v>167</v>
       </c>
       <c r="F71" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G71" s="8" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="H71" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I71" s="8" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="J71" s="7">
         <v>16</v>
@@ -3933,16 +3937,16 @@
         <v>168</v>
       </c>
       <c r="F72" s="9" t="s">
-        <v>210</v>
+        <v>370</v>
       </c>
       <c r="G72" s="10" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H72" s="9" t="s">
-        <v>319</v>
-      </c>
-      <c r="I72" s="10" t="s">
-        <v>372</v>
+        <v>317</v>
+      </c>
+      <c r="I72" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J72" s="9">
         <v>2</v>
@@ -3965,16 +3969,16 @@
         <v>169</v>
       </c>
       <c r="F73" s="7" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G73" s="8" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="H73" s="7" t="s">
-        <v>320</v>
-      </c>
-      <c r="I73" s="8" t="s">
-        <v>372</v>
+        <v>318</v>
+      </c>
+      <c r="I73" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J73" s="7">
         <v>1</v>
@@ -3997,16 +4001,16 @@
         <v>170</v>
       </c>
       <c r="F74" s="9" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G74" s="10" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="H74" s="9" t="s">
-        <v>321</v>
-      </c>
-      <c r="I74" s="10" t="s">
-        <v>372</v>
+        <v>319</v>
+      </c>
+      <c r="I74" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J74" s="9">
         <v>1</v>
@@ -4029,16 +4033,16 @@
         <v>171</v>
       </c>
       <c r="F75" s="7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G75" s="8" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="H75" s="7" t="s">
-        <v>322</v>
-      </c>
-      <c r="I75" s="8" t="s">
-        <v>372</v>
+        <v>320</v>
+      </c>
+      <c r="I75" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J75" s="7">
         <v>1</v>
@@ -4061,16 +4065,16 @@
         <v>172</v>
       </c>
       <c r="F76" s="9" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="G76" s="10" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="H76" s="9" t="s">
-        <v>320</v>
-      </c>
-      <c r="I76" s="10" t="s">
-        <v>372</v>
+        <v>318</v>
+      </c>
+      <c r="I76" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J76" s="9">
         <v>1</v>
@@ -4093,16 +4097,16 @@
         <v>173</v>
       </c>
       <c r="F77" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="G77" s="8" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="H77" s="7" t="s">
-        <v>320</v>
-      </c>
-      <c r="I77" s="8" t="s">
-        <v>372</v>
+        <v>318</v>
+      </c>
+      <c r="I77" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J77" s="7">
         <v>2</v>
@@ -4125,16 +4129,16 @@
         <v>174</v>
       </c>
       <c r="F78" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="G78" s="10" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="H78" s="9" t="s">
-        <v>323</v>
-      </c>
-      <c r="I78" s="10" t="s">
-        <v>372</v>
+        <v>321</v>
+      </c>
+      <c r="I78" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J78" s="9">
         <v>1</v>
@@ -4157,16 +4161,16 @@
         <v>175</v>
       </c>
       <c r="F79" s="7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="G79" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="H79" s="7" t="s">
-        <v>324</v>
-      </c>
-      <c r="I79" s="8" t="s">
-        <v>372</v>
+        <v>322</v>
+      </c>
+      <c r="I79" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="J79" s="7">
         <v>1</v>
@@ -4182,30 +4186,28 @@
       <c r="C80" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D80" s="9" t="s">
+      <c r="D80" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="E80" s="10" t="s">
+      <c r="E80" s="17" t="s">
         <v>176</v>
       </c>
-      <c r="F80" s="9" t="s">
-        <v>218</v>
-      </c>
-      <c r="G80" s="10" t="s">
-        <v>286</v>
-      </c>
-      <c r="H80" s="9" t="s">
-        <v>325</v>
-      </c>
-      <c r="I80" s="10" t="s">
-        <v>333</v>
-      </c>
-      <c r="J80" s="9">
+      <c r="F80" s="16" t="s">
+        <v>217</v>
+      </c>
+      <c r="G80" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="H80" s="16" t="s">
+        <v>323</v>
+      </c>
+      <c r="I80" s="17" t="s">
+        <v>331</v>
+      </c>
+      <c r="J80" s="16">
         <v>1</v>
       </c>
-      <c r="K80" s="15" t="s">
-        <v>333</v>
-      </c>
+      <c r="K80" s="18"/>
     </row>
     <row r="81" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="1"/>
@@ -4222,17 +4224,17 @@
       <c r="E81" s="8" t="s">
         <v>177</v>
       </c>
-      <c r="F81" s="7" t="s">
-        <v>219</v>
+      <c r="F81" s="9" t="s">
+        <v>370</v>
       </c>
       <c r="G81" s="8" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="H81" s="7" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="I81" s="8" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="J81" s="7">
         <v>1</v>
@@ -4255,27 +4257,21 @@
         <v>178</v>
       </c>
       <c r="F82" s="9" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="G82" s="10" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="H82" s="9" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="I82" s="10" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="J82" s="9">
         <v>1</v>
       </c>
       <c r="K82" s="9"/>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="J83">
-        <f>SUM(J3:J82)</f>
-        <v>274</v>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>